<commit_message>
Added code to calculate a tracker acceptance correction
</commit_message>
<xml_diff>
--- a/Sheets/MonteCarloCampaign.xlsx
+++ b/Sheets/MonteCarloCampaign.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10111"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/samuelgrant/Documents/gm2/EDM/Sheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9EA5345-B9C0-274E-BC39-BD8AFC7BD612}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B080B26B-4695-C34A-8C45-FE1772C54129}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="16940" xr2:uid="{5EC16708-1E7D-0544-B394-6DCD03338369}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="37">
   <si>
     <t xml:space="preserve">Date </t>
   </si>
@@ -115,13 +115,43 @@
   </si>
   <si>
     <t>2022-02-14-05-41-40</t>
+  </si>
+  <si>
+    <t>2022-02-17-06-51-28</t>
+  </si>
+  <si>
+    <t>2022-02-17-07-00-32</t>
+  </si>
+  <si>
+    <t>trackTruthTrees.5.root (2956362)</t>
+  </si>
+  <si>
+    <t>2022-02-17-18-24-53</t>
+  </si>
+  <si>
+    <t>2022-02-19-12-42-39</t>
+  </si>
+  <si>
+    <t>2022-02-23-16-06-56</t>
+  </si>
+  <si>
+    <t>2022-02-23-16-07-20</t>
+  </si>
+  <si>
+    <t>2022-02-23-16-07-40</t>
+  </si>
+  <si>
+    <t>2022-02-23-16-10-20</t>
+  </si>
+  <si>
+    <t>Result</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -142,8 +172,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -156,8 +194,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -191,13 +235,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -207,13 +259,19 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -541,31 +599,33 @@
   <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12" style="3" customWidth="1"/>
-    <col min="2" max="2" width="20" style="3" customWidth="1"/>
-    <col min="3" max="3" width="13.5" style="3" customWidth="1"/>
-    <col min="4" max="4" width="11.83203125" style="3" customWidth="1"/>
-    <col min="5" max="5" width="20.5" style="3" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12" style="2" customWidth="1"/>
+    <col min="2" max="2" width="20" style="2" customWidth="1"/>
+    <col min="3" max="3" width="13.5" style="2" customWidth="1"/>
+    <col min="4" max="4" width="11.83203125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="20.5" style="2" customWidth="1"/>
+    <col min="6" max="6" width="28.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="4" t="s">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="1"/>
+      <c r="F1" s="8" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="5">
@@ -583,6 +643,9 @@
       <c r="E2" s="6" t="s">
         <v>5</v>
       </c>
+      <c r="F2" s="7" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="5">
@@ -600,6 +663,7 @@
       <c r="E3" s="6" t="s">
         <v>8</v>
       </c>
+      <c r="F3" s="7"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="5">
@@ -617,6 +681,7 @@
       <c r="E4" s="6" t="s">
         <v>13</v>
       </c>
+      <c r="F4" s="7"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="5">
@@ -634,6 +699,7 @@
       <c r="E5" s="6" t="s">
         <v>14</v>
       </c>
+      <c r="F5" s="7"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="5">
@@ -651,6 +717,7 @@
       <c r="E6" s="6" t="s">
         <v>15</v>
       </c>
+      <c r="F6" s="7"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="5">
@@ -668,6 +735,7 @@
       <c r="E7" s="6" t="s">
         <v>15</v>
       </c>
+      <c r="F7" s="7"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="5">
@@ -680,11 +748,12 @@
         <v>1</v>
       </c>
       <c r="D8" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>18</v>
       </c>
+      <c r="F8" s="7"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="5">
@@ -697,11 +766,12 @@
         <v>1</v>
       </c>
       <c r="D9" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9" s="6" t="s">
         <v>19</v>
       </c>
+      <c r="F9" s="7"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="5">
@@ -714,11 +784,12 @@
         <v>1</v>
       </c>
       <c r="D10" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>23</v>
       </c>
+      <c r="F10" s="7"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="5">
@@ -731,11 +802,12 @@
         <v>1</v>
       </c>
       <c r="D11" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E11" s="6" t="s">
         <v>24</v>
       </c>
+      <c r="F11" s="7"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="5">
@@ -748,336 +820,364 @@
         <v>1</v>
       </c>
       <c r="D12" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>25</v>
       </c>
+      <c r="F12" s="7"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A13" s="7">
+      <c r="A13" s="4">
         <v>44606</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D13" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E13" s="2"/>
+      <c r="C13" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D13" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A14" s="7"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D14" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E14" s="2"/>
+      <c r="A14" s="4">
+        <v>44609</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D14" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D15" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E15" s="2"/>
+      <c r="A15" s="4">
+        <v>44609</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C15" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D15" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D16" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E16" s="2"/>
+      <c r="A16" s="4">
+        <v>44611</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C16" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D16" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D17" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E17" s="2"/>
+      <c r="A17" s="4">
+        <v>44615</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C17" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="D17" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E17" s="1"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D18" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E18" s="2"/>
+      <c r="A18" s="1"/>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="D18" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E18" s="1"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A19" s="2"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D19" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E19" s="2"/>
+      <c r="A19" s="1"/>
+      <c r="B19" s="1"/>
+      <c r="C19" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="D19" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E19" s="1"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A20" s="2"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D20" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E20" s="2"/>
+      <c r="A20" s="1"/>
+      <c r="B20" s="1"/>
+      <c r="C20" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="D20" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E20" s="1"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A21" s="2"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D21" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E21" s="2"/>
+      <c r="A21" s="1"/>
+      <c r="B21" s="1"/>
+      <c r="C21" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="D21" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E21" s="1"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A22" s="2"/>
-      <c r="B22" s="2"/>
-      <c r="C22" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D22" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E22" s="2"/>
+      <c r="A22" s="1"/>
+      <c r="B22" s="1"/>
+      <c r="C22" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="D22" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E22" s="1"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A23" s="2"/>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D23" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E23" s="2"/>
+      <c r="A23" s="1"/>
+      <c r="B23" s="1"/>
+      <c r="C23" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="D23" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E23" s="1"/>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A24" s="2"/>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D24" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E24" s="2"/>
+      <c r="A24" s="1"/>
+      <c r="B24" s="1"/>
+      <c r="C24" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="D24" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E24" s="1"/>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A25" s="2"/>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D25" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E25" s="2"/>
+      <c r="A25" s="1"/>
+      <c r="B25" s="1"/>
+      <c r="C25" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="D25" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E25" s="1"/>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A26" s="2"/>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D26" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E26" s="2"/>
+      <c r="A26" s="1"/>
+      <c r="B26" s="1"/>
+      <c r="C26" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="D26" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E26" s="1"/>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A27" s="2"/>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D27" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E27" s="2"/>
+      <c r="A27" s="1"/>
+      <c r="B27" s="1"/>
+      <c r="C27" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="D27" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E27" s="1"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A28" s="2"/>
-      <c r="B28" s="2"/>
-      <c r="C28" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D28" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E28" s="2"/>
+      <c r="A28" s="1"/>
+      <c r="B28" s="1"/>
+      <c r="C28" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="D28" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E28" s="1"/>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A29" s="2"/>
-      <c r="B29" s="2"/>
-      <c r="C29" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D29" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E29" s="2"/>
+      <c r="A29" s="1"/>
+      <c r="B29" s="1"/>
+      <c r="C29" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="D29" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E29" s="1"/>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A30" s="2"/>
-      <c r="B30" s="2"/>
-      <c r="C30" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D30" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E30" s="2"/>
+      <c r="A30" s="1"/>
+      <c r="B30" s="1"/>
+      <c r="C30" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="D30" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E30" s="1"/>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A31" s="2"/>
-      <c r="B31" s="2"/>
-      <c r="C31" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D31" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E31" s="2"/>
+      <c r="A31" s="1"/>
+      <c r="B31" s="1"/>
+      <c r="C31" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="D31" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E31" s="1"/>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A32" s="2"/>
-      <c r="B32" s="2"/>
-      <c r="C32" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D32" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E32" s="2"/>
+      <c r="A32" s="1"/>
+      <c r="B32" s="1"/>
+      <c r="C32" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="D32" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E32" s="1"/>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A33" s="2"/>
-      <c r="B33" s="2"/>
-      <c r="C33" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D33" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E33" s="2"/>
+      <c r="A33" s="1"/>
+      <c r="B33" s="1"/>
+      <c r="C33" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="D33" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E33" s="1"/>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A34" s="2"/>
-      <c r="B34" s="2"/>
-      <c r="C34" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D34" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E34" s="2"/>
+      <c r="A34" s="1"/>
+      <c r="B34" s="1"/>
+      <c r="C34" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="D34" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E34" s="1"/>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A35" s="2"/>
-      <c r="B35" s="2"/>
-      <c r="C35" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D35" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E35" s="2"/>
+      <c r="A35" s="1"/>
+      <c r="B35" s="1"/>
+      <c r="C35" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="D35" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E35" s="1"/>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A36" s="2"/>
-      <c r="B36" s="2"/>
-      <c r="C36" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D36" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E36" s="2"/>
+      <c r="A36" s="1"/>
+      <c r="B36" s="1"/>
+      <c r="C36" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="D36" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E36" s="1"/>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A37" s="2"/>
-      <c r="B37" s="2"/>
-      <c r="C37" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D37" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E37" s="2"/>
+      <c r="A37" s="1"/>
+      <c r="B37" s="1"/>
+      <c r="C37" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="D37" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E37" s="1"/>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A38" s="2"/>
-      <c r="B38" s="2"/>
-      <c r="C38" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D38" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E38" s="2"/>
+      <c r="A38" s="1"/>
+      <c r="B38" s="1"/>
+      <c r="C38" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="D38" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E38" s="1"/>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A39" s="2"/>
-      <c r="B39" s="2"/>
-      <c r="C39" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D39" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E39" s="2"/>
+      <c r="A39" s="1"/>
+      <c r="B39" s="1"/>
+      <c r="C39" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="D39" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E39" s="1"/>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A40" s="2"/>
-      <c r="B40" s="2"/>
-      <c r="C40" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D40" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E40" s="2"/>
+      <c r="A40" s="1"/>
+      <c r="B40" s="1"/>
+      <c r="C40" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="D40" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E40" s="1"/>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A41" s="2"/>
-      <c r="B41" s="2"/>
-      <c r="C41" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D41" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E41" s="2"/>
+      <c r="A41" s="1"/>
+      <c r="B41" s="1"/>
+      <c r="C41" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="D41" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E41" s="1"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="F2:F12"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Tidied things up (a bit)
</commit_message>
<xml_diff>
--- a/Sheets/MonteCarloCampaign.xlsx
+++ b/Sheets/MonteCarloCampaign.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10520"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10708"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/samuelgrant/Documents/gm2/EDM/Sheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C9B66C1-D76C-FF42-A09A-DF2E41F4651B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D444030-570D-6547-AFCD-775B7B4D897D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="520" windowWidth="28040" windowHeight="16940" xr2:uid="{5EC16708-1E7D-0544-B394-6DCD03338369}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{5EC16708-1E7D-0544-B394-6DCD03338369}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="86">
   <si>
     <t xml:space="preserve">Date </t>
   </si>
@@ -254,13 +254,55 @@
   </si>
   <si>
     <t>2022-03-24-21-38-22</t>
+  </si>
+  <si>
+    <t>Events</t>
+  </si>
+  <si>
+    <t>Raw</t>
+  </si>
+  <si>
+    <t>Cuts</t>
+  </si>
+  <si>
+    <t>Jobs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Events </t>
+  </si>
+  <si>
+    <t>Events / submission</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vertices / submission </t>
+  </si>
+  <si>
+    <t>Vertices / event</t>
+  </si>
+  <si>
+    <t>Events / vertex</t>
+  </si>
+  <si>
+    <t>Cuts vertices / submission</t>
+  </si>
+  <si>
+    <t>Events / vertex (raw)</t>
+  </si>
+  <si>
+    <t>Events / vertex (cuts)</t>
+  </si>
+  <si>
+    <t>On Tape</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.000%"/>
+  </numFmts>
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -289,6 +331,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -310,7 +359,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -454,11 +503,32 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -521,13 +591,29 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Per cent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -847,7 +933,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32DC9D9F-763E-3C49-967B-5A1EE4155DD8}">
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:R41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12" style="2" customWidth="1"/>
@@ -857,10 +943,16 @@
     <col min="5" max="5" width="20.5" style="2" customWidth="1"/>
     <col min="6" max="6" width="28.6640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.1640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -882,11 +974,14 @@
       <c r="G1" s="5" t="s">
         <v>50</v>
       </c>
+      <c r="H1" s="5" t="s">
+        <v>73</v>
+      </c>
       <c r="I1" s="6" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2" s="14">
         <v>44593</v>
       </c>
@@ -902,18 +997,30 @@
       <c r="E2" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="23" t="s">
+      <c r="F2" s="26" t="s">
         <v>51</v>
       </c>
-      <c r="G2" s="23">
+      <c r="G2" s="26">
         <v>5484331</v>
       </c>
-      <c r="I2" s="7">
-        <f>SUM(G2:G41)</f>
-        <v>8058825</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H2">
+        <v>1000</v>
+      </c>
+      <c r="I2" s="24">
+        <v>50000</v>
+      </c>
+      <c r="J2">
+        <f>I2*H2</f>
+        <v>50000000</v>
+      </c>
+      <c r="K2">
+        <v>5</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A3" s="16">
         <v>44599</v>
       </c>
@@ -929,10 +1036,40 @@
       <c r="E3" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="F3" s="23"/>
-      <c r="G3" s="23"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F3" s="26"/>
+      <c r="G3" s="26"/>
+      <c r="H3">
+        <v>1000</v>
+      </c>
+      <c r="I3" s="24">
+        <v>50000</v>
+      </c>
+      <c r="K3" t="s">
+        <v>74</v>
+      </c>
+      <c r="L3" s="22">
+        <v>5484331</v>
+      </c>
+      <c r="M3" s="23">
+        <f>L3/(20000)</f>
+        <v>274.21654999999998</v>
+      </c>
+      <c r="N3" s="22">
+        <f>20*1000*50000</f>
+        <v>1000000000</v>
+      </c>
+      <c r="P3" t="s">
+        <v>74</v>
+      </c>
+      <c r="Q3">
+        <v>10671380</v>
+      </c>
+      <c r="R3">
+        <f>Q3*L9</f>
+        <v>1945794300.1616788</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A4" s="16">
         <v>44601</v>
       </c>
@@ -948,10 +1085,32 @@
       <c r="E4" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="F4" s="23"/>
-      <c r="G4" s="23"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F4" s="26"/>
+      <c r="G4" s="26"/>
+      <c r="H4">
+        <v>1000</v>
+      </c>
+      <c r="I4" s="24">
+        <v>50000</v>
+      </c>
+      <c r="K4" t="s">
+        <v>75</v>
+      </c>
+      <c r="L4" s="22">
+        <v>2366239</v>
+      </c>
+      <c r="P4" t="s">
+        <v>75</v>
+      </c>
+      <c r="Q4">
+        <v>4603005</v>
+      </c>
+      <c r="R4" s="22">
+        <f>Q4*L10</f>
+        <v>1945283211.036586</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A5" s="16">
         <v>44601</v>
       </c>
@@ -967,10 +1126,23 @@
       <c r="E5" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="F5" s="23"/>
-      <c r="G5" s="23"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F5" s="26"/>
+      <c r="G5" s="26"/>
+      <c r="H5">
+        <v>1000</v>
+      </c>
+      <c r="I5" s="24">
+        <v>50000</v>
+      </c>
+      <c r="K5" t="s">
+        <v>76</v>
+      </c>
+      <c r="L5">
+        <f>SUM(H2:H21)</f>
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A6" s="16">
         <v>44602</v>
       </c>
@@ -986,10 +1158,23 @@
       <c r="E6" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="F6" s="23"/>
-      <c r="G6" s="23"/>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F6" s="26"/>
+      <c r="G6" s="26"/>
+      <c r="H6">
+        <v>1000</v>
+      </c>
+      <c r="I6" s="24">
+        <v>50000</v>
+      </c>
+      <c r="K6" t="s">
+        <v>77</v>
+      </c>
+      <c r="L6" s="22">
+        <f>J2*COUNT(I2:I21)</f>
+        <v>1000000000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A7" s="16">
         <v>44602</v>
       </c>
@@ -1005,10 +1190,16 @@
       <c r="E7" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="F7" s="23"/>
-      <c r="G7" s="23"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F7" s="26"/>
+      <c r="G7" s="26"/>
+      <c r="H7">
+        <v>1000</v>
+      </c>
+      <c r="I7" s="24">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A8" s="16">
         <v>44603</v>
       </c>
@@ -1024,10 +1215,16 @@
       <c r="E8" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="F8" s="23"/>
-      <c r="G8" s="23"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F8" s="26"/>
+      <c r="G8" s="26"/>
+      <c r="H8">
+        <v>1000</v>
+      </c>
+      <c r="I8" s="24">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A9" s="16">
         <v>44603</v>
       </c>
@@ -1043,10 +1240,23 @@
       <c r="E9" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="F9" s="23"/>
-      <c r="G9" s="23"/>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F9" s="26"/>
+      <c r="G9" s="26"/>
+      <c r="H9">
+        <v>1000</v>
+      </c>
+      <c r="I9" s="24">
+        <v>50000</v>
+      </c>
+      <c r="K9" t="s">
+        <v>83</v>
+      </c>
+      <c r="L9" s="23">
+        <f>L6/L3</f>
+        <v>182.33764519318765</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A10" s="16">
         <v>44604</v>
       </c>
@@ -1062,10 +1272,23 @@
       <c r="E10" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="F10" s="23"/>
-      <c r="G10" s="23"/>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F10" s="26"/>
+      <c r="G10" s="26"/>
+      <c r="H10">
+        <v>1000</v>
+      </c>
+      <c r="I10" s="24">
+        <v>50000</v>
+      </c>
+      <c r="K10" t="s">
+        <v>84</v>
+      </c>
+      <c r="L10" s="23">
+        <f>L6/L4</f>
+        <v>422.61157896560746</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A11" s="16">
         <v>44605</v>
       </c>
@@ -1081,10 +1304,16 @@
       <c r="E11" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="F11" s="23"/>
-      <c r="G11" s="23"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F11" s="26"/>
+      <c r="G11" s="26"/>
+      <c r="H11">
+        <v>1000</v>
+      </c>
+      <c r="I11" s="24">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A12" s="18">
         <v>44605</v>
       </c>
@@ -1100,10 +1329,16 @@
       <c r="E12" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="F12" s="23"/>
-      <c r="G12" s="23"/>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F12" s="26"/>
+      <c r="G12" s="26"/>
+      <c r="H12">
+        <v>1000</v>
+      </c>
+      <c r="I12" s="24">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A13" s="19">
         <v>44606</v>
       </c>
@@ -1119,10 +1354,17 @@
       <c r="E13" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="F13" s="23"/>
-      <c r="G13" s="23"/>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F13" s="26"/>
+      <c r="G13" s="26"/>
+      <c r="H13">
+        <v>1000</v>
+      </c>
+      <c r="I13" s="24">
+        <v>50000</v>
+      </c>
+      <c r="M13" s="23"/>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A14" s="10">
         <v>44609</v>
       </c>
@@ -1138,10 +1380,16 @@
       <c r="E14" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="F14" s="23"/>
-      <c r="G14" s="23"/>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F14" s="26"/>
+      <c r="G14" s="26"/>
+      <c r="H14">
+        <v>1000</v>
+      </c>
+      <c r="I14" s="24">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A15" s="10">
         <v>44609</v>
       </c>
@@ -1157,10 +1405,16 @@
       <c r="E15" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="F15" s="23"/>
-      <c r="G15" s="23"/>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F15" s="26"/>
+      <c r="G15" s="26"/>
+      <c r="H15">
+        <v>1000</v>
+      </c>
+      <c r="I15" s="24">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A16" s="10">
         <v>44611</v>
       </c>
@@ -1176,10 +1430,23 @@
       <c r="E16" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="F16" s="23"/>
-      <c r="G16" s="23"/>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F16" s="26"/>
+      <c r="G16" s="26"/>
+      <c r="H16">
+        <v>1000</v>
+      </c>
+      <c r="I16" s="24">
+        <v>50000</v>
+      </c>
+      <c r="K16" t="s">
+        <v>78</v>
+      </c>
+      <c r="L16" s="22">
+        <f>H2*I2</f>
+        <v>50000000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" s="10">
         <v>44615</v>
       </c>
@@ -1195,10 +1462,23 @@
       <c r="E17" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="F17" s="23"/>
-      <c r="G17" s="23"/>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F17" s="26"/>
+      <c r="G17" s="26"/>
+      <c r="H17">
+        <v>1000</v>
+      </c>
+      <c r="I17" s="24">
+        <v>50000</v>
+      </c>
+      <c r="K17" t="s">
+        <v>79</v>
+      </c>
+      <c r="L17" s="22" t="e">
+        <f>L3/L7</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" s="10">
         <v>44616</v>
       </c>
@@ -1214,10 +1494,16 @@
       <c r="E18" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="F18" s="23"/>
-      <c r="G18" s="23"/>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F18" s="26"/>
+      <c r="G18" s="26"/>
+      <c r="H18">
+        <v>1000</v>
+      </c>
+      <c r="I18" s="24">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" s="10">
         <v>44617</v>
       </c>
@@ -1233,10 +1519,23 @@
       <c r="E19" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="F19" s="23"/>
-      <c r="G19" s="23"/>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F19" s="26"/>
+      <c r="G19" s="26"/>
+      <c r="H19">
+        <v>1000</v>
+      </c>
+      <c r="I19" s="24">
+        <v>50000</v>
+      </c>
+      <c r="K19" t="s">
+        <v>80</v>
+      </c>
+      <c r="L19" s="25" t="e">
+        <f>L17/L16</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" s="10">
         <v>44619</v>
       </c>
@@ -1252,10 +1551,23 @@
       <c r="E20" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="F20" s="23"/>
-      <c r="G20" s="23"/>
-    </row>
-    <row r="21" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="F20" s="26"/>
+      <c r="G20" s="26"/>
+      <c r="H20">
+        <v>1000</v>
+      </c>
+      <c r="I20" s="24">
+        <v>50000</v>
+      </c>
+      <c r="K20" t="s">
+        <v>81</v>
+      </c>
+      <c r="L20" s="23" t="e">
+        <f>L16/L17</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21" s="12">
         <v>44620</v>
       </c>
@@ -1271,10 +1583,20 @@
       <c r="E21" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="F21" s="23"/>
-      <c r="G21" s="23"/>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F21" s="26"/>
+      <c r="G21" s="26"/>
+      <c r="H21">
+        <v>1000</v>
+      </c>
+      <c r="I21" s="24">
+        <v>50000</v>
+      </c>
+      <c r="J21" s="22">
+        <f>I21*H21*COUNT(H2:H21)</f>
+        <v>1000000000</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22" s="8">
         <v>44621</v>
       </c>
@@ -1290,14 +1612,25 @@
       <c r="E22" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="F22" s="23" t="s">
+      <c r="F22" s="27" t="s">
         <v>69</v>
       </c>
-      <c r="G22" s="23">
-        <v>2574494</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G22" s="28"/>
+      <c r="H22">
+        <v>1000</v>
+      </c>
+      <c r="I22" s="24">
+        <v>50000</v>
+      </c>
+      <c r="K22" t="s">
+        <v>82</v>
+      </c>
+      <c r="L22" s="22" t="e">
+        <f>L4/L7</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" s="10">
         <v>44622</v>
       </c>
@@ -1313,10 +1646,23 @@
       <c r="E23" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="F23" s="23"/>
-      <c r="G23" s="23"/>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F23" s="29"/>
+      <c r="G23" s="30"/>
+      <c r="H23">
+        <v>1000</v>
+      </c>
+      <c r="I23" s="24">
+        <v>50000</v>
+      </c>
+      <c r="K23" t="s">
+        <v>81</v>
+      </c>
+      <c r="L23" s="22" t="e">
+        <f>L16/L22</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" s="10">
         <v>44623</v>
       </c>
@@ -1332,10 +1678,16 @@
       <c r="E24" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="F24" s="23"/>
-      <c r="G24" s="23"/>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F24" s="29"/>
+      <c r="G24" s="30"/>
+      <c r="H24">
+        <v>1000</v>
+      </c>
+      <c r="I24" s="24">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" s="10">
         <v>44629</v>
       </c>
@@ -1351,10 +1703,16 @@
       <c r="E25" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="F25" s="23"/>
-      <c r="G25" s="23"/>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F25" s="29"/>
+      <c r="G25" s="30"/>
+      <c r="H25">
+        <v>1000</v>
+      </c>
+      <c r="I25" s="24">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A26" s="10">
         <v>44633</v>
       </c>
@@ -1370,10 +1728,16 @@
       <c r="E26" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="F26" s="23"/>
-      <c r="G26" s="23"/>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F26" s="29"/>
+      <c r="G26" s="30"/>
+      <c r="H26">
+        <v>1000</v>
+      </c>
+      <c r="I26" s="24">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A27" s="10">
         <v>44634</v>
       </c>
@@ -1389,10 +1753,16 @@
       <c r="E27" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="F27" s="23"/>
-      <c r="G27" s="23"/>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F27" s="29"/>
+      <c r="G27" s="30"/>
+      <c r="H27">
+        <v>1000</v>
+      </c>
+      <c r="I27" s="24">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" s="10">
         <v>44634</v>
       </c>
@@ -1408,10 +1778,19 @@
       <c r="E28" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="F28" s="23"/>
-      <c r="G28" s="23"/>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F28" s="29"/>
+      <c r="G28" s="30"/>
+      <c r="H28">
+        <v>1000</v>
+      </c>
+      <c r="I28" s="24">
+        <v>50000</v>
+      </c>
+      <c r="K28" s="22">
+        <v>4000000000</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A29" s="10">
         <v>44635</v>
       </c>
@@ -1427,10 +1806,20 @@
       <c r="E29" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="F29" s="23"/>
-      <c r="G29" s="23"/>
-    </row>
-    <row r="30" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="F29" s="29"/>
+      <c r="G29" s="30"/>
+      <c r="H29">
+        <v>1000</v>
+      </c>
+      <c r="I29" s="24">
+        <v>50000</v>
+      </c>
+      <c r="K29">
+        <f>(H30*I30)</f>
+        <v>50000000</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A30" s="12">
         <v>44636</v>
       </c>
@@ -1446,10 +1835,20 @@
       <c r="E30" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="F30" s="23"/>
-      <c r="G30" s="23"/>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F30" s="29"/>
+      <c r="G30" s="30"/>
+      <c r="H30">
+        <v>1000</v>
+      </c>
+      <c r="I30" s="24">
+        <v>50000</v>
+      </c>
+      <c r="K30" s="23">
+        <f>K28/K29</f>
+        <v>80</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A31" s="20">
         <v>44637</v>
       </c>
@@ -1465,10 +1864,14 @@
       <c r="E31" s="21" t="s">
         <v>70</v>
       </c>
-      <c r="F31" s="22"/>
-      <c r="G31" s="22"/>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F31" s="29"/>
+      <c r="G31" s="30"/>
+      <c r="H31" s="22">
+        <f>SUM(H22:H30)*SUM(I22:I30)</f>
+        <v>4050000000</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A32" s="19">
         <v>44638</v>
       </c>
@@ -1484,8 +1887,12 @@
       <c r="E32" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="F32" s="22"/>
-      <c r="G32" s="22"/>
+      <c r="F32" s="29"/>
+      <c r="G32" s="30"/>
+      <c r="H32" s="7" t="e">
+        <f>H31/SUM(G22)</f>
+        <v>#DIV/0!</v>
+      </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" s="19">
@@ -1503,8 +1910,8 @@
       <c r="E33" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="F33" s="22"/>
-      <c r="G33" s="22"/>
+      <c r="F33" s="29"/>
+      <c r="G33" s="30"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" s="1"/>
@@ -1595,11 +2002,10 @@
       <c r="E41" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="3">
     <mergeCell ref="F2:F21"/>
     <mergeCell ref="G2:G21"/>
-    <mergeCell ref="F22:F30"/>
-    <mergeCell ref="G22:G30"/>
+    <mergeCell ref="F22:G33"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>